<commit_message>
updated data w 11.21th and attempting run
</commit_message>
<xml_diff>
--- a/inst/extdata/meteostat_data/export (33).xlsx
+++ b/inst/extdata/meteostat_data/export (33).xlsx
@@ -1,19 +1,318 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c770e11f011a8c48/DKM/Stats_R/R/MartysGas/inst/extdata/meteostat_data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_4C75EF5A7964FF18F55B1250EA3161BAD3501258" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{597F57A7-80CC-4F1C-B80A-7CC95ABC28DB}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="25100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+  <si>
+    <t>tavg</t>
+  </si>
+  <si>
+    <t>tmin</t>
+  </si>
+  <si>
+    <t>tmax</t>
+  </si>
+  <si>
+    <t>prcp</t>
+  </si>
+  <si>
+    <t>snow</t>
+  </si>
+  <si>
+    <t>wdir</t>
+  </si>
+  <si>
+    <t>wspd</t>
+  </si>
+  <si>
+    <t>wpgt</t>
+  </si>
+  <si>
+    <t>pres</t>
+  </si>
+  <si>
+    <t>tsun</t>
+  </si>
+  <si>
+    <t>2025-01-01</t>
+  </si>
+  <si>
+    <t>2025-01-02</t>
+  </si>
+  <si>
+    <t>2025-01-03</t>
+  </si>
+  <si>
+    <t>2025-01-04</t>
+  </si>
+  <si>
+    <t>2025-01-05</t>
+  </si>
+  <si>
+    <t>2025-01-06</t>
+  </si>
+  <si>
+    <t>2025-01-07</t>
+  </si>
+  <si>
+    <t>2025-01-08</t>
+  </si>
+  <si>
+    <t>2025-01-09</t>
+  </si>
+  <si>
+    <t>2025-01-10</t>
+  </si>
+  <si>
+    <t>2025-01-11</t>
+  </si>
+  <si>
+    <t>2025-01-12</t>
+  </si>
+  <si>
+    <t>2025-01-13</t>
+  </si>
+  <si>
+    <t>2025-01-14</t>
+  </si>
+  <si>
+    <t>2025-01-15</t>
+  </si>
+  <si>
+    <t>2025-01-16</t>
+  </si>
+  <si>
+    <t>2025-01-17</t>
+  </si>
+  <si>
+    <t>2025-01-18</t>
+  </si>
+  <si>
+    <t>2025-01-19</t>
+  </si>
+  <si>
+    <t>2025-01-20</t>
+  </si>
+  <si>
+    <t>2025-01-21</t>
+  </si>
+  <si>
+    <t>2025-01-22</t>
+  </si>
+  <si>
+    <t>2025-01-23</t>
+  </si>
+  <si>
+    <t>2025-01-24</t>
+  </si>
+  <si>
+    <t>2025-01-25</t>
+  </si>
+  <si>
+    <t>2025-01-26</t>
+  </si>
+  <si>
+    <t>2025-01-27</t>
+  </si>
+  <si>
+    <t>2025-01-28</t>
+  </si>
+  <si>
+    <t>2025-01-29</t>
+  </si>
+  <si>
+    <t>2025-01-30</t>
+  </si>
+  <si>
+    <t>2025-01-31</t>
+  </si>
+  <si>
+    <t>2025-02-01</t>
+  </si>
+  <si>
+    <t>2025-02-02</t>
+  </si>
+  <si>
+    <t>2025-02-03</t>
+  </si>
+  <si>
+    <t>2025-02-04</t>
+  </si>
+  <si>
+    <t>2025-02-05</t>
+  </si>
+  <si>
+    <t>2025-02-06</t>
+  </si>
+  <si>
+    <t>2025-02-07</t>
+  </si>
+  <si>
+    <t>2025-02-08</t>
+  </si>
+  <si>
+    <t>2025-02-09</t>
+  </si>
+  <si>
+    <t>2025-02-10</t>
+  </si>
+  <si>
+    <t>2025-02-11</t>
+  </si>
+  <si>
+    <t>2025-02-12</t>
+  </si>
+  <si>
+    <t>2025-02-13</t>
+  </si>
+  <si>
+    <t>2025-02-14</t>
+  </si>
+  <si>
+    <t>2025-02-15</t>
+  </si>
+  <si>
+    <t>2025-02-16</t>
+  </si>
+  <si>
+    <t>2025-02-17</t>
+  </si>
+  <si>
+    <t>2025-02-18</t>
+  </si>
+  <si>
+    <t>2025-02-19</t>
+  </si>
+  <si>
+    <t>2025-02-20</t>
+  </si>
+  <si>
+    <t>2025-02-21</t>
+  </si>
+  <si>
+    <t>2025-02-22</t>
+  </si>
+  <si>
+    <t>2025-02-23</t>
+  </si>
+  <si>
+    <t>2025-02-24</t>
+  </si>
+  <si>
+    <t>2025-02-25</t>
+  </si>
+  <si>
+    <t>2025-02-26</t>
+  </si>
+  <si>
+    <t>2025-02-27</t>
+  </si>
+  <si>
+    <t>2025-02-28</t>
+  </si>
+  <si>
+    <t>2025-03-01</t>
+  </si>
+  <si>
+    <t>2025-03-02</t>
+  </si>
+  <si>
+    <t>2025-03-03</t>
+  </si>
+  <si>
+    <t>2025-03-04</t>
+  </si>
+  <si>
+    <t>2025-03-05</t>
+  </si>
+  <si>
+    <t>2025-03-06</t>
+  </si>
+  <si>
+    <t>2025-03-07</t>
+  </si>
+  <si>
+    <t>2025-03-08</t>
+  </si>
+  <si>
+    <t>2025-03-09</t>
+  </si>
+  <si>
+    <t>2025-03-10</t>
+  </si>
+  <si>
+    <t>2025-03-11</t>
+  </si>
+  <si>
+    <t>2025-03-12</t>
+  </si>
+  <si>
+    <t>2025-03-13</t>
+  </si>
+  <si>
+    <t>2025-03-14</t>
+  </si>
+  <si>
+    <t>2025-03-15</t>
+  </si>
+  <si>
+    <t>2025-03-16</t>
+  </si>
+  <si>
+    <t>2025-03-17</t>
+  </si>
+  <si>
+    <t>2025-03-18</t>
+  </si>
+  <si>
+    <t>2025-03-19</t>
+  </si>
+  <si>
+    <t>2025-03-20</t>
+  </si>
+  <si>
+    <t>2025-03-21</t>
+  </si>
+  <si>
+    <t>2025-03-22</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -43,13 +342,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -374,47 +681,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K82"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>tavg</v>
-      </c>
-      <c r="C1" t="str">
-        <v>tmin</v>
-      </c>
-      <c r="D1" t="str">
-        <v>tmax</v>
-      </c>
-      <c r="E1" t="str">
-        <v>prcp</v>
-      </c>
-      <c r="F1" t="str">
-        <v>snow</v>
-      </c>
-      <c r="G1" t="str">
-        <v>wdir</v>
-      </c>
-      <c r="H1" t="str">
-        <v>wspd</v>
-      </c>
-      <c r="I1" t="str">
-        <v>wpgt</v>
-      </c>
-      <c r="J1" t="str">
-        <v>pres</v>
-      </c>
-      <c r="K1" t="str">
-        <v>tsun</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2025-01-01</v>
+    <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
       </c>
       <c r="B2">
         <v>-3.1</v>
@@ -441,9 +746,9 @@
         <v>1030.7</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2025-01-02</v>
+    <row r="3" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>11</v>
       </c>
       <c r="B3">
         <v>-1.7</v>
@@ -470,9 +775,9 @@
         <v>1018.9</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2025-01-03</v>
+    <row r="4" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
       </c>
       <c r="B4">
         <v>1.7</v>
@@ -481,7 +786,7 @@
         <v>-0.4</v>
       </c>
       <c r="D4">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E4">
         <v>1.4</v>
@@ -490,7 +795,7 @@
         <v>297</v>
       </c>
       <c r="H4">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="I4">
         <v>39</v>
@@ -499,9 +804,9 @@
         <v>1015.6</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2025-01-04</v>
+    <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>13</v>
       </c>
       <c r="B5">
         <v>1.2</v>
@@ -528,15 +833,15 @@
         <v>1022.7</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2025-01-05</v>
+    <row r="6" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
       </c>
       <c r="B6">
         <v>-1.8</v>
       </c>
       <c r="C6">
-        <v>-4.4</v>
+        <v>-4.4000000000000004</v>
       </c>
       <c r="D6">
         <v>0.9</v>
@@ -557,9 +862,9 @@
         <v>1016.9</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>2025-01-06</v>
+    <row r="7" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>15</v>
       </c>
       <c r="B7">
         <v>5.2</v>
@@ -586,15 +891,15 @@
         <v>1008.5</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>2025-01-07</v>
+    <row r="8" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>16</v>
       </c>
       <c r="B8">
         <v>8.9</v>
       </c>
       <c r="C8">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D8">
         <v>13.7</v>
@@ -615,9 +920,9 @@
         <v>1009.1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>2025-01-08</v>
+    <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
       </c>
       <c r="B9">
         <v>6.1</v>
@@ -644,9 +949,9 @@
         <v>1012.1</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>2025-01-09</v>
+    <row r="10" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>18</v>
       </c>
       <c r="B10">
         <v>8.6</v>
@@ -673,12 +978,12 @@
         <v>1009.4</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>2025-01-10</v>
+    <row r="11" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>19</v>
       </c>
       <c r="B11">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="C11">
         <v>0.6</v>
@@ -702,9 +1007,9 @@
         <v>1013.7</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>2025-01-11</v>
+    <row r="12" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>20</v>
       </c>
       <c r="B12">
         <v>0.3</v>
@@ -713,7 +1018,7 @@
         <v>-4.3</v>
       </c>
       <c r="D12">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E12">
         <v>0.1</v>
@@ -731,9 +1036,9 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>2025-01-12</v>
+    <row r="13" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>21</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -757,12 +1062,12 @@
         <v>64.8</v>
       </c>
       <c r="J13">
-        <v>1024.4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>2025-01-13</v>
+        <v>1024.4000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>22</v>
       </c>
       <c r="B14">
         <v>0.8</v>
@@ -789,15 +1094,15 @@
         <v>1036.7</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>2025-01-14</v>
+    <row r="15" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>23</v>
       </c>
       <c r="B15">
-        <v>-1.1</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="C15">
-        <v>-4.6</v>
+        <v>-4.5999999999999996</v>
       </c>
       <c r="D15">
         <v>2.7</v>
@@ -818,9 +1123,9 @@
         <v>1037.5</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>2025-01-15</v>
+    <row r="16" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>24</v>
       </c>
       <c r="B16">
         <v>-1</v>
@@ -847,9 +1152,9 @@
         <v>1028.8</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>2025-01-16</v>
+    <row r="17" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>25</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -873,12 +1178,12 @@
         <v>11</v>
       </c>
       <c r="J17">
-        <v>1038.6</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>2025-01-17</v>
+        <v>1038.5999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>26</v>
       </c>
       <c r="B18">
         <v>-0.2</v>
@@ -905,9 +1210,9 @@
         <v>1042.2</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>2025-01-18</v>
+    <row r="19" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>27</v>
       </c>
       <c r="B19">
         <v>-0.6</v>
@@ -931,12 +1236,12 @@
         <v>14</v>
       </c>
       <c r="J19">
-        <v>1037.9</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>2025-01-19</v>
+        <v>1037.9000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>28</v>
       </c>
       <c r="B20">
         <v>-2.5</v>
@@ -963,9 +1268,9 @@
         <v>1033.2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>2025-01-20</v>
+    <row r="21" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>29</v>
       </c>
       <c r="B21">
         <v>-2.5</v>
@@ -989,18 +1294,18 @@
         <v>14</v>
       </c>
       <c r="J21">
-        <v>1029.9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>2025-01-21</v>
+        <v>1029.9000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>30</v>
       </c>
       <c r="B22">
         <v>-1.8</v>
       </c>
       <c r="C22">
-        <v>-2.3</v>
+        <v>-2.2999999999999998</v>
       </c>
       <c r="D22">
         <v>-1.3</v>
@@ -1021,9 +1326,9 @@
         <v>1022.5</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>2025-01-22</v>
+    <row r="23" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>31</v>
       </c>
       <c r="B23">
         <v>-1.4</v>
@@ -1050,9 +1355,9 @@
         <v>1019.6</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>2025-01-23</v>
+    <row r="24" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>32</v>
       </c>
       <c r="B24">
         <v>0.9</v>
@@ -1064,7 +1369,7 @@
         <v>2.5</v>
       </c>
       <c r="E24">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G24">
         <v>41</v>
@@ -1079,18 +1384,18 @@
         <v>1014.8</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>2025-01-24</v>
+    <row r="25" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>33</v>
       </c>
       <c r="B25">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C25">
         <v>1.8</v>
       </c>
       <c r="D25">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -1108,15 +1413,15 @@
         <v>1018.6</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>2025-01-25</v>
+    <row r="26" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>34</v>
       </c>
       <c r="B26">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="C26">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="D26">
         <v>9.6</v>
@@ -1137,9 +1442,9 @@
         <v>1020.8</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>2025-01-26</v>
+    <row r="27" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>35</v>
       </c>
       <c r="B27">
         <v>7.2</v>
@@ -1166,12 +1471,12 @@
         <v>1015.9</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>2025-01-27</v>
+    <row r="28" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>36</v>
       </c>
       <c r="B28">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="C28">
         <v>3.8</v>
@@ -1195,9 +1500,9 @@
         <v>1012.1</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>2025-01-28</v>
+    <row r="29" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>37</v>
       </c>
       <c r="B29">
         <v>10.5</v>
@@ -1224,9 +1529,9 @@
         <v>1006.7</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>2025-01-29</v>
+    <row r="30" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>38</v>
       </c>
       <c r="B30">
         <v>8</v>
@@ -1253,9 +1558,9 @@
         <v>1013.7</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>2025-01-30</v>
+    <row r="31" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>39</v>
       </c>
       <c r="B31">
         <v>6.4</v>
@@ -1282,15 +1587,15 @@
         <v>1020.5</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>2025-01-31</v>
+    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>40</v>
       </c>
       <c r="B32">
         <v>6.7</v>
       </c>
       <c r="C32">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D32">
         <v>11.1</v>
@@ -1311,12 +1616,12 @@
         <v>1024.5</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>2025-02-01</v>
+    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>41</v>
       </c>
       <c r="B33">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1337,12 +1642,12 @@
         <v>23</v>
       </c>
       <c r="J33">
-        <v>1031.1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>2025-02-02</v>
+        <v>1031.0999999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>42</v>
       </c>
       <c r="B34">
         <v>3.1</v>
@@ -1366,18 +1671,18 @@
         <v>17</v>
       </c>
       <c r="J34">
-        <v>1026.4</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>2025-02-03</v>
+        <v>1026.4000000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>43</v>
       </c>
       <c r="B35">
         <v>1.7</v>
       </c>
       <c r="C35">
-        <v>-2.2</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="D35">
         <v>5.6</v>
@@ -1389,7 +1694,7 @@
         <v>73</v>
       </c>
       <c r="H35">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="I35">
         <v>12</v>
@@ -1398,15 +1703,15 @@
         <v>1028.2</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>2025-02-04</v>
+    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>44</v>
       </c>
       <c r="B36">
-        <v>-1.1</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="C36">
-        <v>-5.1</v>
+        <v>-5.0999999999999996</v>
       </c>
       <c r="D36">
         <v>4.3</v>
@@ -1427,9 +1732,9 @@
         <v>1032.7</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>2025-02-05</v>
+    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>45</v>
       </c>
       <c r="B37">
         <v>1.4</v>
@@ -1456,9 +1761,9 @@
         <v>1034.5</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>2025-02-06</v>
+    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>46</v>
       </c>
       <c r="B38">
         <v>1.7</v>
@@ -1476,18 +1781,18 @@
         <v>67</v>
       </c>
       <c r="H38">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I38">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="J38">
         <v>1036.8</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>2025-02-07</v>
+    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>47</v>
       </c>
       <c r="B39">
         <v>1.7</v>
@@ -1514,9 +1819,9 @@
         <v>1036.8</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>2025-02-08</v>
+    <row r="40" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>48</v>
       </c>
       <c r="B40">
         <v>1.6</v>
@@ -1543,9 +1848,9 @@
         <v>1035.8</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>2025-02-09</v>
+    <row r="41" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>49</v>
       </c>
       <c r="B41">
         <v>1.5</v>
@@ -1572,9 +1877,9 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>2025-02-10</v>
+    <row r="42" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>50</v>
       </c>
       <c r="B42">
         <v>1.9</v>
@@ -1598,18 +1903,18 @@
         <v>14</v>
       </c>
       <c r="J42">
-        <v>1030.9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>2025-02-11</v>
+        <v>1030.9000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>51</v>
       </c>
       <c r="B43">
         <v>0.1</v>
       </c>
       <c r="C43">
-        <v>-4.6</v>
+        <v>-4.5999999999999996</v>
       </c>
       <c r="D43">
         <v>6.1</v>
@@ -1630,9 +1935,9 @@
         <v>1031.3</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>2025-02-12</v>
+    <row r="44" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>52</v>
       </c>
       <c r="B44">
         <v>0.7</v>
@@ -1650,7 +1955,7 @@
         <v>111</v>
       </c>
       <c r="H44">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I44">
         <v>30</v>
@@ -1659,9 +1964,9 @@
         <v>1028.3</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>2025-02-13</v>
+    <row r="45" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>53</v>
       </c>
       <c r="B45">
         <v>-0.3</v>
@@ -1688,12 +1993,12 @@
         <v>1021.1</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>2025-02-14</v>
+    <row r="46" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>54</v>
       </c>
       <c r="B46">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="C46">
         <v>0.6</v>
@@ -1717,12 +2022,12 @@
         <v>1016.9</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>2025-02-15</v>
+    <row r="47" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>55</v>
       </c>
       <c r="B47">
-        <v>-1.1</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="C47">
         <v>-4.8</v>
@@ -1737,7 +2042,7 @@
         <v>222</v>
       </c>
       <c r="H47">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I47">
         <v>28</v>
@@ -1746,9 +2051,9 @@
         <v>1023.4</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>2025-02-16</v>
+    <row r="48" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>56</v>
       </c>
       <c r="B48">
         <v>-3.1</v>
@@ -1775,9 +2080,9 @@
         <v>1022.6</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>2025-02-17</v>
+    <row r="49" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>57</v>
       </c>
       <c r="B49">
         <v>-1.8</v>
@@ -1786,7 +2091,7 @@
         <v>-5.7</v>
       </c>
       <c r="D49">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -1804,9 +2109,9 @@
         <v>1025.8</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>2025-02-18</v>
+    <row r="50" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>58</v>
       </c>
       <c r="B50">
         <v>-1.8</v>
@@ -1833,15 +2138,15 @@
         <v>1028.2</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>2025-02-19</v>
+    <row r="51" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>59</v>
       </c>
       <c r="B51">
         <v>-2.8</v>
       </c>
       <c r="C51">
-        <v>-8.2</v>
+        <v>-8.1999999999999993</v>
       </c>
       <c r="D51">
         <v>2.7</v>
@@ -1862,9 +2167,9 @@
         <v>1034.2</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>2025-02-20</v>
+    <row r="52" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>60</v>
       </c>
       <c r="B52">
         <v>-2.4</v>
@@ -1888,12 +2193,12 @@
         <v>20</v>
       </c>
       <c r="J52">
-        <v>1035.4</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>2025-02-21</v>
+        <v>1035.4000000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>61</v>
       </c>
       <c r="B53">
         <v>-1.6</v>
@@ -1920,9 +2225,9 @@
         <v>1036.3</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>2025-02-22</v>
+    <row r="54" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>62</v>
       </c>
       <c r="B54">
         <v>-0.2</v>
@@ -1940,7 +2245,7 @@
         <v>106</v>
       </c>
       <c r="H54">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="I54">
         <v>32</v>
@@ -1949,9 +2254,9 @@
         <v>1032.7</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>2025-02-23</v>
+    <row r="55" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>63</v>
       </c>
       <c r="B55">
         <v>1.7</v>
@@ -1969,7 +2274,7 @@
         <v>111</v>
       </c>
       <c r="H55">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I55">
         <v>15</v>
@@ -1978,9 +2283,9 @@
         <v>1031.7</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>2025-02-24</v>
+    <row r="56" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>64</v>
       </c>
       <c r="B56">
         <v>3.2</v>
@@ -2004,12 +2309,12 @@
         <v>15</v>
       </c>
       <c r="J56">
-        <v>1029.4</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>2025-02-25</v>
+        <v>1029.4000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>65</v>
       </c>
       <c r="B57">
         <v>3.6</v>
@@ -2036,9 +2341,9 @@
         <v>1023.1</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>2025-02-26</v>
+    <row r="58" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>66</v>
       </c>
       <c r="B58">
         <v>3.5</v>
@@ -2050,7 +2355,7 @@
         <v>4.7</v>
       </c>
       <c r="E58">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="G58">
         <v>44</v>
@@ -2065,18 +2370,18 @@
         <v>1018.7</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2025-02-27</v>
+    <row r="59" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>67</v>
       </c>
       <c r="B59">
         <v>6.6</v>
       </c>
       <c r="C59">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D59">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="E59">
         <v>7.1</v>
@@ -2094,9 +2399,9 @@
         <v>1017.8</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2025-02-28</v>
+    <row r="60" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>68</v>
       </c>
       <c r="B60">
         <v>6.6</v>
@@ -2114,7 +2419,7 @@
         <v>295</v>
       </c>
       <c r="H60">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="I60">
         <v>33</v>
@@ -2123,9 +2428,9 @@
         <v>1020.7</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2025-03-01</v>
+    <row r="61" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>69</v>
       </c>
       <c r="B61">
         <v>6</v>
@@ -2152,18 +2457,18 @@
         <v>1026.2</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2025-03-02</v>
+    <row r="62" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>70</v>
       </c>
       <c r="B62">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="C62">
         <v>0.9</v>
       </c>
       <c r="D62">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -2178,12 +2483,12 @@
         <v>20</v>
       </c>
       <c r="J62">
-        <v>1029.6</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2025-03-03</v>
+        <v>1029.5999999999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>71</v>
       </c>
       <c r="B63">
         <v>4.2</v>
@@ -2192,7 +2497,7 @@
         <v>-0.9</v>
       </c>
       <c r="D63">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -2210,9 +2515,9 @@
         <v>1029.3</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2025-03-04</v>
+    <row r="64" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>72</v>
       </c>
       <c r="B64">
         <v>5.4</v>
@@ -2239,9 +2544,9 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>2025-03-05</v>
+    <row r="65" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>73</v>
       </c>
       <c r="B65">
         <v>7.6</v>
@@ -2259,18 +2564,18 @@
         <v>144</v>
       </c>
       <c r="H65">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I65">
         <v>17</v>
       </c>
       <c r="J65">
-        <v>1028.9</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>2025-03-06</v>
+        <v>1028.9000000000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>74</v>
       </c>
       <c r="B66">
         <v>10.3</v>
@@ -2279,7 +2584,7 @@
         <v>2</v>
       </c>
       <c r="D66">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -2294,12 +2599,12 @@
         <v>23</v>
       </c>
       <c r="J66">
-        <v>1027.6</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <v>2025-03-07</v>
+        <v>1027.5999999999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>75</v>
       </c>
       <c r="B67">
         <v>11.3</v>
@@ -2308,7 +2613,7 @@
         <v>3.6</v>
       </c>
       <c r="D67">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -2326,9 +2631,9 @@
         <v>1022.8</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>2025-03-08</v>
+    <row r="68" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>76</v>
       </c>
       <c r="B68">
         <v>12.1</v>
@@ -2346,7 +2651,7 @@
         <v>68</v>
       </c>
       <c r="H68">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I68">
         <v>23</v>
@@ -2355,9 +2660,9 @@
         <v>1017.3</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>2025-03-09</v>
+    <row r="69" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>77</v>
       </c>
       <c r="B69">
         <v>11.7</v>
@@ -2384,9 +2689,9 @@
         <v>1012.2</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v>2025-03-10</v>
+    <row r="70" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>78</v>
       </c>
       <c r="B70">
         <v>12.3</v>
@@ -2404,7 +2709,7 @@
         <v>162</v>
       </c>
       <c r="H70">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="I70">
         <v>35</v>
@@ -2413,15 +2718,15 @@
         <v>1007.2</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>2025-03-11</v>
+    <row r="71" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>79</v>
       </c>
       <c r="B71">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="C71">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="D71">
         <v>11.7</v>
@@ -2442,9 +2747,9 @@
         <v>1005.4</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="str">
-        <v>2025-03-12</v>
+    <row r="72" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>80</v>
       </c>
       <c r="B72">
         <v>11.8</v>
@@ -2453,7 +2758,7 @@
         <v>5.4</v>
       </c>
       <c r="D72">
-        <v>18.6</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="E72">
         <v>0</v>
@@ -2471,9 +2776,9 @@
         <v>1002.5</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="str">
-        <v>2025-03-13</v>
+    <row r="73" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>81</v>
       </c>
       <c r="B73">
         <v>12.2</v>
@@ -2500,9 +2805,9 @@
         <v>996.4</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <v>2025-03-14</v>
+    <row r="74" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>82</v>
       </c>
       <c r="B74">
         <v>10.1</v>
@@ -2529,9 +2834,9 @@
         <v>1005.7</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="str">
-        <v>2025-03-15</v>
+    <row r="75" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>83</v>
       </c>
       <c r="B75">
         <v>9.6</v>
@@ -2549,18 +2854,18 @@
         <v>5.9</v>
       </c>
       <c r="I75">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="J75">
         <v>1010.7</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="str">
-        <v>2025-03-16</v>
+    <row r="76" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>84</v>
       </c>
       <c r="B76">
-        <v>8.7</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="C76">
         <v>6.7</v>
@@ -2575,15 +2880,15 @@
         <v>5.7</v>
       </c>
       <c r="I76">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="J76">
         <v>1016.3</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="str">
-        <v>2025-03-17</v>
+    <row r="77" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>85</v>
       </c>
       <c r="B77">
         <v>7.7</v>
@@ -2607,9 +2912,9 @@
         <v>1020.7</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="str">
-        <v>2025-03-18</v>
+    <row r="78" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>86</v>
       </c>
       <c r="B78">
         <v>5.7</v>
@@ -2633,9 +2938,9 @@
         <v>1029.7</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="str">
-        <v>2025-03-19</v>
+    <row r="79" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>87</v>
       </c>
       <c r="B79">
         <v>6.4</v>
@@ -2653,15 +2958,15 @@
         <v>7.3</v>
       </c>
       <c r="I79">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="J79">
-        <v>1031.6</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="str">
-        <v>2025-03-20</v>
+        <v>1031.5999999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>88</v>
       </c>
       <c r="B80">
         <v>6.5</v>
@@ -2682,18 +2987,18 @@
         <v>42.6</v>
       </c>
       <c r="J80">
-        <v>1028.4</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="str">
-        <v>2025-03-21</v>
+        <v>1028.4000000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>89</v>
       </c>
       <c r="B81">
         <v>7.7</v>
       </c>
       <c r="C81">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D81">
         <v>12.9</v>
@@ -2711,9 +3016,9 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="str">
-        <v>2025-03-22</v>
+    <row r="82" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>90</v>
       </c>
       <c r="B82">
         <v>8.6</v>
@@ -2738,8 +3043,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K82"/>
+    <ignoredError sqref="A2:K82 B1:K1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>